<commit_message>
Advance retriever + some improvements to improve context_recall
</commit_message>
<xml_diff>
--- a/RiskHalo_Certification_Challenge/data/Weekly_Trade_Data_Uploads/Week_22_Trade_data.xlsx
+++ b/RiskHalo_Certification_Challenge/data/Weekly_Trade_Data_Uploads/Week_22_Trade_data.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1A6A866-914F-4F08-A79C-D6BD41038E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Weekly_Data" sheetId="1" r:id="rId1"/>
@@ -112,9 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -522,49 +520,49 @@
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="A3">
         <v>209</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="1">
         <v>45960</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3">
         <v>75</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3">
         <v>137.44999999999999</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3">
         <v>10308.75</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3">
         <v>75</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3">
         <v>167.55</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3">
         <v>12566.25</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3">
         <v>0</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3">
         <v>2257.5</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3">
         <v>69.81</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3">
         <v>2187.69</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3">
         <v>2257.5</v>
       </c>
     </row>

</xml_diff>